<commit_message>
refactor(web): reescribe index y developers con arco narrativo, tabs, acordeón, timeline y Quality Layer
- index.html: hero con actividad live, sección antes/después, timeline 'Un día con Hermes', héroes en tabs desktop / acordeón mobile, carta como blockquote, impacto sin números inventados.
- developers.html: hero corto, arquitectura con Eval Loop, perfiles en tabs/acordeón, sección Quality Layer con diagrama, demo code real, conexiones y workshop simplificado.
- Actualiza README.md y TODOS.md con el nuevo scope.
- Regenera screenshots desktop/mobile.
- Verifica demo Tesorero y build del dashboard.
</commit_message>
<xml_diff>
--- a/data/sample_gastos.xlsx
+++ b/data/sample_gastos.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Ingresos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Gastos Fijos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Gastos Variables" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Proveedores" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ingresos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gastos Fijos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gastos Variables" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proveedores" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>